<commit_message>
sync: 2026-04-17 08:00 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dr-cleugo/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dr-cleugo/campaigns/data.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="119">
   <si>
     <t>ID da Campanha</t>
   </si>
@@ -60,37 +60,52 @@
     <t>Observações</t>
   </si>
   <si>
+    <t>120245734861770249</t>
+  </si>
+  <si>
+    <t>[Syra] Emagrecimento Retargeting Morno [Formulário Instantâneo] [CBO]</t>
+  </si>
+  <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
+    <t>OUTCOME_LEADS</t>
+  </si>
+  <si>
+    <t>15/04/2026</t>
+  </si>
+  <si>
+    <t>✅ Ativa</t>
+  </si>
+  <si>
+    <t>120245734151500249</t>
+  </si>
+  <si>
+    <t>[Syra] Emagrecimento Retargeting Morno [Formulário Instantâneo] [ABO]</t>
+  </si>
+  <si>
+    <t>PAUSED</t>
+  </si>
+  <si>
+    <t>⏸️ Pausada</t>
+  </si>
+  <si>
     <t>120243740011460249</t>
   </si>
   <si>
     <t>[Syra] Dra Gabrielle - Emagrecimento [São Paulo] [Formulário Instantâneo] [CBO]</t>
   </si>
   <si>
-    <t>PAUSED</t>
-  </si>
-  <si>
-    <t>OUTCOME_LEADS</t>
-  </si>
-  <si>
     <t>19/03/2026</t>
   </si>
   <si>
-    <t>⏸️ Pausada</t>
-  </si>
-  <si>
     <t>120243183154170249</t>
   </si>
   <si>
     <t>[Syra] Dra Gabrielle - Emagrecimento [Formulário Instantâneo] [CBO]</t>
   </si>
   <si>
-    <t>ACTIVE</t>
-  </si>
-  <si>
     <t>10/03/2026</t>
-  </si>
-  <si>
-    <t>✅ Ativa</t>
   </si>
   <si>
     <t>120242484578140249</t>
@@ -396,12 +411,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF99"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFFFFF99"/>
       </patternFill>
     </fill>
   </fills>
@@ -768,7 +783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -848,7 +863,7 @@
         <v>18</v>
       </c>
       <c r="E2" s="8">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>19</v>
@@ -895,10 +910,10 @@
         <v>18</v>
       </c>
       <c r="E3" s="1">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -925,28 +940,28 @@
         <v>0</v>
       </c>
       <c r="O3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="8">
+        <v>20</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="8">
-        <v>6</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="G4" s="6">
         <v>0</v>
       </c>
@@ -972,27 +987,27 @@
         <v>0</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E5" s="1">
+        <v>35</v>
+      </c>
+      <c r="F5" t="s">
         <v>30</v>
-      </c>
-      <c r="F5" t="s">
-        <v>32</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1024,19 +1039,19 @@
     </row>
     <row r="6" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>28</v>
-      </c>
       <c r="E6" s="8">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>34</v>
@@ -1066,7 +1081,7 @@
         <v>0</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1076,14 +1091,14 @@
       <c r="B7" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>17</v>
+      <c r="C7" s="10" t="s">
+        <v>23</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E7" s="1">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
         <v>37</v>
@@ -1113,7 +1128,7 @@
         <v>0</v>
       </c>
       <c r="O7" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1121,20 +1136,20 @@
         <v>38</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" s="8">
-        <v>0</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>41</v>
-      </c>
       <c r="G8" s="6">
         <v>0</v>
       </c>
@@ -1160,28 +1175,28 @@
         <v>0</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="1">
+        <v>15</v>
+      </c>
+      <c r="F9" t="s">
         <v>42</v>
       </c>
-      <c r="B9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="1">
-        <v>0</v>
-      </c>
-      <c r="F9" t="s">
-        <v>44</v>
-      </c>
       <c r="G9">
         <v>0</v>
       </c>
@@ -1207,28 +1222,28 @@
         <v>0</v>
       </c>
       <c r="O9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="E10" s="8">
+        <v>0</v>
+      </c>
+      <c r="F10" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="8">
-        <v>0</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>47</v>
-      </c>
       <c r="G10" s="6">
         <v>0</v>
       </c>
@@ -1254,28 +1269,28 @@
         <v>0</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
         <v>48</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0</v>
+      </c>
+      <c r="F11" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="1">
-        <v>0</v>
-      </c>
-      <c r="F11" t="s">
-        <v>50</v>
-      </c>
       <c r="G11">
         <v>0</v>
       </c>
@@ -1301,28 +1316,28 @@
         <v>0</v>
       </c>
       <c r="O11" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="C12" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="8">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="8">
-        <v>0</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>53</v>
-      </c>
       <c r="G12" s="6">
         <v>0</v>
       </c>
@@ -1348,28 +1363,28 @@
         <v>0</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" t="s">
         <v>54</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0</v>
-      </c>
-      <c r="F13" t="s">
-        <v>56</v>
-      </c>
       <c r="G13">
         <v>0</v>
       </c>
@@ -1395,28 +1410,28 @@
         <v>0</v>
       </c>
       <c r="O13" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="8">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E14" s="8">
-        <v>0</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>59</v>
-      </c>
       <c r="G14" s="6">
         <v>0</v>
       </c>
@@ -1442,28 +1457,28 @@
         <v>0</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" t="s">
         <v>60</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" t="s">
-        <v>40</v>
-      </c>
-      <c r="E15" s="1">
-        <v>0</v>
-      </c>
-      <c r="F15" t="s">
-        <v>62</v>
-      </c>
       <c r="G15">
         <v>0</v>
       </c>
@@ -1489,28 +1504,28 @@
         <v>0</v>
       </c>
       <c r="O15" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="8">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E16" s="8">
-        <v>0</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>65</v>
-      </c>
       <c r="G16" s="6">
         <v>0</v>
       </c>
@@ -1536,28 +1551,28 @@
         <v>0</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" t="s">
         <v>66</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0</v>
+      </c>
+      <c r="F17" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" t="s">
-        <v>40</v>
-      </c>
-      <c r="E17" s="1">
-        <v>30</v>
-      </c>
-      <c r="F17" t="s">
-        <v>68</v>
-      </c>
       <c r="G17">
         <v>0</v>
       </c>
@@ -1583,28 +1598,28 @@
         <v>0</v>
       </c>
       <c r="O17" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="8">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E18" s="8">
-        <v>0</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>71</v>
-      </c>
       <c r="G18" s="6">
         <v>0</v>
       </c>
@@ -1630,28 +1645,28 @@
         <v>0</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" t="s">
         <v>72</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="1">
+        <v>30</v>
+      </c>
+      <c r="F19" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D19" t="s">
-        <v>40</v>
-      </c>
-      <c r="E19" s="1">
-        <v>0</v>
-      </c>
-      <c r="F19" t="s">
-        <v>74</v>
-      </c>
       <c r="G19">
         <v>0</v>
       </c>
@@ -1677,28 +1692,28 @@
         <v>0</v>
       </c>
       <c r="O19" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="C20" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" s="8">
+        <v>0</v>
+      </c>
+      <c r="F20" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E20" s="8">
-        <v>0</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>77</v>
-      </c>
       <c r="G20" s="6">
         <v>0</v>
       </c>
@@ -1724,28 +1739,28 @@
         <v>0</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" t="s">
         <v>78</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0</v>
+      </c>
+      <c r="F21" t="s">
         <v>79</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E21" s="1">
-        <v>10</v>
-      </c>
-      <c r="F21" t="s">
-        <v>80</v>
-      </c>
       <c r="G21">
         <v>0</v>
       </c>
@@ -1771,28 +1786,28 @@
         <v>0</v>
       </c>
       <c r="O21" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="C22" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="8">
+        <v>0</v>
+      </c>
+      <c r="F22" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E22" s="8">
-        <v>0</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>83</v>
-      </c>
       <c r="G22" s="6">
         <v>0</v>
       </c>
@@ -1818,28 +1833,28 @@
         <v>0</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>83</v>
+      </c>
+      <c r="B23" t="s">
         <v>84</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D23" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" s="1">
+        <v>10</v>
+      </c>
+      <c r="F23" t="s">
         <v>85</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D23" t="s">
-        <v>40</v>
-      </c>
-      <c r="E23" s="1">
-        <v>0</v>
-      </c>
-      <c r="F23" t="s">
-        <v>86</v>
-      </c>
       <c r="G23">
         <v>0</v>
       </c>
@@ -1865,28 +1880,28 @@
         <v>0</v>
       </c>
       <c r="O23" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="C24" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E24" s="8">
+        <v>0</v>
+      </c>
+      <c r="F24" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E24" s="8">
-        <v>25</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>89</v>
-      </c>
       <c r="G24" s="6">
         <v>0</v>
       </c>
@@ -1912,28 +1927,28 @@
         <v>0</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" t="s">
         <v>90</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0</v>
+      </c>
+      <c r="F25" t="s">
         <v>91</v>
       </c>
-      <c r="C25" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D25" t="s">
-        <v>92</v>
-      </c>
-      <c r="E25" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="F25" t="s">
-        <v>93</v>
-      </c>
       <c r="G25">
         <v>0</v>
       </c>
@@ -1959,28 +1974,28 @@
         <v>0</v>
       </c>
       <c r="O25" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26" s="8">
+        <v>25</v>
+      </c>
+      <c r="F26" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B26" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E26" s="8">
-        <v>13</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>96</v>
-      </c>
       <c r="G26" s="6">
         <v>0</v>
       </c>
@@ -2006,54 +2021,148 @@
         <v>0</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>95</v>
+      </c>
+      <c r="B27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27" t="s">
         <v>97</v>
       </c>
-      <c r="B27" t="s">
+      <c r="E27" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="F27" t="s">
         <v>98</v>
       </c>
-      <c r="C27" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27" s="1">
+        <v>0</v>
+      </c>
+      <c r="J27" s="1">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27" s="2">
+        <v>0</v>
+      </c>
+      <c r="N27" s="1">
+        <v>0</v>
+      </c>
+      <c r="O27" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E27" s="1">
+      <c r="B28" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E28" s="8">
+        <v>13</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="G28" s="6">
+        <v>0</v>
+      </c>
+      <c r="H28" s="6">
+        <v>0</v>
+      </c>
+      <c r="I28" s="8">
+        <v>0</v>
+      </c>
+      <c r="J28" s="8">
+        <v>0</v>
+      </c>
+      <c r="K28" s="6">
+        <v>0</v>
+      </c>
+      <c r="L28" s="6">
+        <v>0</v>
+      </c>
+      <c r="M28" s="9">
+        <v>0</v>
+      </c>
+      <c r="N28" s="8">
+        <v>0</v>
+      </c>
+      <c r="O28" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>102</v>
+      </c>
+      <c r="B29" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D29" t="s">
+        <v>104</v>
+      </c>
+      <c r="E29" s="1">
         <v>6.5</v>
       </c>
-      <c r="F27" t="s">
-        <v>100</v>
-      </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="H27">
-        <v>0</v>
-      </c>
-      <c r="I27" s="1">
-        <v>0</v>
-      </c>
-      <c r="J27" s="1">
-        <v>0</v>
-      </c>
-      <c r="K27">
-        <v>0</v>
-      </c>
-      <c r="L27">
-        <v>0</v>
-      </c>
-      <c r="M27" s="2">
-        <v>0</v>
-      </c>
-      <c r="N27" s="1">
-        <v>0</v>
-      </c>
-      <c r="O27" t="s">
-        <v>20</v>
+      <c r="F29" t="s">
+        <v>105</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29" s="1">
+        <v>0</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="M29" s="2">
+        <v>0</v>
+      </c>
+      <c r="N29" s="1">
+        <v>0</v>
+      </c>
+      <c r="O29" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -2082,13 +2191,13 @@
   <sheetData>
     <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -2097,7 +2206,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>6</v>
@@ -2112,30 +2221,30 @@
         <v>9</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -2153,7 +2262,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2180,19 +2289,19 @@
   <sheetData>
     <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>6</v>
@@ -2210,24 +2319,24 @@
         <v>2</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -2242,10 +2351,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="K2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync: 2026-04-22 08:00 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dr-cleugo/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dr-cleugo/campaigns/data.xlsx
@@ -863,7 +863,7 @@
         <v>18</v>
       </c>
       <c r="E2" s="8">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>19</v>
@@ -1004,7 +1004,7 @@
         <v>18</v>
       </c>
       <c r="E5" s="1">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
sync: 2026-04-24 08:00 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dr-cleugo/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dr-cleugo/campaigns/data.xlsx
@@ -863,7 +863,7 @@
         <v>18</v>
       </c>
       <c r="E2" s="8">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>19</v>
@@ -1004,7 +1004,7 @@
         <v>18</v>
       </c>
       <c r="E5" s="1">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
sync: 2026-04-28 08:00 — atualizacao automatica diaria
</commit_message>
<xml_diff>
--- a/meu-projeto/docs/clientes/dr-cleugo/campaigns/data.xlsx
+++ b/meu-projeto/docs/clientes/dr-cleugo/campaigns/data.xlsx
@@ -102,7 +102,7 @@
     <t>120243183154170249</t>
   </si>
   <si>
-    <t>[Syra] Dra Gabrielle - Emagrecimento [Formulário Instantâneo] [CBO]</t>
+    <t>[Syra] Emagrecimento Publico Frio [Formulário Instantâneo] [ABO]</t>
   </si>
   <si>
     <t>10/03/2026</t>
@@ -863,7 +863,7 @@
         <v>18</v>
       </c>
       <c r="E2" s="8">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>19</v>
@@ -1004,7 +1004,7 @@
         <v>18</v>
       </c>
       <c r="E5" s="1">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F5" t="s">
         <v>30</v>

</xml_diff>